<commit_message>
Mise à jour des données d'inscription
</commit_message>
<xml_diff>
--- a/fichier_eleves/J1.xlsx
+++ b/fichier_eleves/J1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="229">
   <si>
     <t>Identifications</t>
   </si>
@@ -64,6 +64,9 @@
     <t xml:space="preserve">Session : </t>
   </si>
   <si>
+    <t>Session A</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -83,6 +86,9 @@
     </r>
   </si>
   <si>
+    <t>Doe</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -102,7 +108,13 @@
     </r>
   </si>
   <si>
+    <t>John</t>
+  </si>
+  <si>
     <t>Date de l'évaluation :</t>
+  </si>
+  <si>
+    <t>2024-12-31</t>
   </si>
   <si>
     <t>Lieu de l'évaluation (entreprise ou centre de formation) :</t>
@@ -2954,7 +2966,9 @@
       <c r="A5" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="16"/>
+      <c r="B5" s="16" t="s">
+        <v>8</v>
+      </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17"/>
@@ -2962,9 +2976,11 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="20"/>
+        <v>9</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>10</v>
+      </c>
       <c r="C6" s="21"/>
       <c r="D6" s="21"/>
       <c r="E6" s="21"/>
@@ -2972,9 +2988,11 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="23"/>
+        <v>11</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>12</v>
+      </c>
       <c r="C7" s="21"/>
       <c r="D7" s="21"/>
       <c r="E7" s="21"/>
@@ -2982,9 +3000,11 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="24"/>
+        <v>13</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>14</v>
+      </c>
       <c r="C8" s="25"/>
       <c r="D8" s="25"/>
       <c r="E8" s="25"/>
@@ -2992,7 +3012,7 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B9" s="28" t="s">
         <v>6</v>
@@ -3012,7 +3032,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -3030,7 +3050,7 @@
     </row>
     <row r="13" ht="24.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -3040,107 +3060,107 @@
     </row>
     <row r="14" ht="25.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="40" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B14" s="41" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C14" s="42" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D14" s="43" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E14" s="44" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F14" s="45" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" ht="25.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="46" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B15" s="47" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C15" s="48" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D15" s="49" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E15" s="50"/>
       <c r="F15" s="45" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" ht="25.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="46" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B16" s="47" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C16" s="48" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D16" s="49" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E16" s="50" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F16" s="45" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" ht="25.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="46" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B17" s="47" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D17" s="49" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E17" s="47"/>
       <c r="F17" s="45" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" ht="25.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="46" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B18" s="47" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D18" s="49" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E18" s="47"/>
       <c r="F18" s="45" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" ht="25.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="46" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B19" s="47" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C19" s="48" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D19" s="51"/>
       <c r="E19" s="52"/>
@@ -3156,7 +3176,7 @@
     </row>
     <row r="21" ht="14.25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="57" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B21" s="58"/>
       <c r="C21" s="58"/>
@@ -3166,7 +3186,7 @@
     </row>
     <row r="22" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -3176,271 +3196,271 @@
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="61" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B23" s="62"/>
       <c r="C23" s="63" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D23" s="64" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E23" s="62"/>
       <c r="F23" s="65"/>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="66" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B24" s="67"/>
       <c r="C24" s="68"/>
       <c r="D24" s="69" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E24" s="67"/>
       <c r="F24" s="70" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="66" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B25" s="67"/>
       <c r="C25" s="68"/>
       <c r="D25" s="69" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E25" s="67"/>
       <c r="F25" s="70" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="66" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B26" s="67"/>
       <c r="C26" s="68"/>
       <c r="D26" s="69" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E26" s="67"/>
       <c r="F26" s="70" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="66" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B27" s="67"/>
       <c r="C27" s="68" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D27" s="69" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E27" s="67"/>
       <c r="F27" s="70"/>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="66" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B28" s="67"/>
       <c r="C28" s="68" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D28" s="69" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E28" s="67"/>
       <c r="F28" s="70" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="66" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B29" s="67"/>
       <c r="C29" s="68"/>
       <c r="D29" s="69" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E29" s="67"/>
       <c r="F29" s="70"/>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="66" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B30" s="67"/>
       <c r="C30" s="68"/>
       <c r="D30" s="69" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E30" s="67"/>
       <c r="F30" s="70"/>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="66" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B31" s="67"/>
       <c r="C31" s="68"/>
       <c r="D31" s="69" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E31" s="67"/>
       <c r="F31" s="70"/>
     </row>
     <row r="32" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="66" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B32" s="67"/>
       <c r="C32" s="68"/>
       <c r="D32" s="69" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E32" s="67"/>
       <c r="F32" s="70"/>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="66" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B33" s="67"/>
       <c r="C33" s="68"/>
       <c r="D33" s="69" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E33" s="67"/>
       <c r="F33" s="70"/>
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="66" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B34" s="67"/>
       <c r="C34" s="71"/>
       <c r="D34" s="72" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E34" s="72"/>
       <c r="F34" s="70"/>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="66" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B35" s="67"/>
       <c r="C35" s="68" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D35" s="73" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E35" s="74"/>
       <c r="F35" s="70" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="75" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B36" s="76"/>
       <c r="C36" s="68" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D36" s="76" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E36" s="76"/>
       <c r="F36" s="70"/>
     </row>
     <row r="37" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="66" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B37" s="67"/>
       <c r="C37" s="77"/>
       <c r="D37" s="73" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E37" s="74"/>
       <c r="F37" s="70"/>
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="66" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B38" s="67"/>
       <c r="C38" s="78"/>
       <c r="D38" s="73" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E38" s="74"/>
       <c r="F38" s="70"/>
     </row>
     <row r="39" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="79" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B39" s="72"/>
       <c r="C39" s="78" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D39" s="73" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E39" s="74"/>
       <c r="F39" s="70"/>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="79" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B40" s="72"/>
       <c r="C40" s="78"/>
       <c r="D40" s="73" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E40" s="74"/>
       <c r="F40" s="70"/>
     </row>
     <row r="41" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="79" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B41" s="72"/>
       <c r="C41" s="78" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D41" s="73" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E41" s="74"/>
       <c r="F41" s="70"/>
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:6" s="60" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="80" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B42" s="81"/>
       <c r="C42" s="82"/>
       <c r="D42" s="83" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E42" s="84"/>
       <c r="F42" s="85"/>
     </row>
     <row r="43" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="86" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B43" s="87"/>
       <c r="C43" s="87"/>
@@ -3576,7 +3596,7 @@
       <c r="I1" s="104"/>
       <c r="J1" s="60"/>
       <c r="K1" s="105" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" ht="31.7" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -3593,14 +3613,14 @@
     </row>
     <row r="3" ht="13.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="113" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B3" s="114"/>
       <c r="C3" s="115" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E3" s="117">
         <v>0</v>
@@ -3615,7 +3635,7 @@
         <v>3</v>
       </c>
       <c r="K3" s="119" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -3650,16 +3670,16 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="126" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B5" s="127" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C5" s="128" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D5" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E5" s="129"/>
       <c r="F5" s="130"/>
@@ -3704,10 +3724,10 @@
       <c r="A6" s="131"/>
       <c r="B6" s="132"/>
       <c r="C6" s="133" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D6" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E6" s="129"/>
       <c r="F6" s="134"/>
@@ -3750,16 +3770,16 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="126" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B7" s="127" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C7" s="136" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D7" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E7" s="129"/>
       <c r="F7" s="134"/>
@@ -3804,10 +3824,10 @@
       <c r="A8" s="131"/>
       <c r="B8" s="132"/>
       <c r="C8" s="137" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D8" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E8" s="129"/>
       <c r="F8" s="134"/>
@@ -3850,16 +3870,16 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="126" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B9" s="127" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C9" s="138" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D9" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E9" s="129"/>
       <c r="F9" s="134"/>
@@ -3904,10 +3924,10 @@
       <c r="A10" s="131"/>
       <c r="B10" s="132"/>
       <c r="C10" s="138" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D10" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E10" s="129"/>
       <c r="F10" s="134"/>
@@ -3950,16 +3970,16 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="126" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B11" s="127" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C11" s="138" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D11" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E11" s="129"/>
       <c r="F11" s="134"/>
@@ -4004,10 +4024,10 @@
       <c r="A12" s="131"/>
       <c r="B12" s="132"/>
       <c r="C12" s="138" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D12" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E12" s="129"/>
       <c r="F12" s="134"/>
@@ -4050,16 +4070,16 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="126" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B13" s="127" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C13" s="139" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D13" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E13" s="129"/>
       <c r="F13" s="134"/>
@@ -4104,10 +4124,10 @@
       <c r="A14" s="131"/>
       <c r="B14" s="140"/>
       <c r="C14" s="141" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D14" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E14" s="129"/>
       <c r="F14" s="142"/>
@@ -4155,7 +4175,7 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="145" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B15" s="146"/>
       <c r="C15" s="146"/>
@@ -4197,28 +4217,28 @@
     </row>
     <row r="16" ht="25.5" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="126" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B16" s="127" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C16" s="148" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D16" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E16" s="129" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F16" s="130" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G16" s="130" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I16" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4260,10 +4280,10 @@
       <c r="A17" s="131"/>
       <c r="B17" s="132"/>
       <c r="C17" s="136" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D17" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E17" s="129"/>
       <c r="F17" s="134"/>
@@ -4306,16 +4326,16 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="126" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B18" s="127" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C18" s="89" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D18" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E18" s="129"/>
       <c r="F18" s="134"/>
@@ -4360,22 +4380,22 @@
       <c r="A19" s="131"/>
       <c r="B19" s="132"/>
       <c r="C19" s="133" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D19" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E19" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F19" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G19" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H19" s="135" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I19" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4415,16 +4435,16 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="126" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B20" s="127" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C20" s="133" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D20" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E20" s="129"/>
       <c r="F20" s="134"/>
@@ -4469,22 +4489,22 @@
       <c r="A21" s="131"/>
       <c r="B21" s="132"/>
       <c r="C21" s="133" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D21" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E21" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F21" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G21" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H21" s="135" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I21" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4520,28 +4540,28 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="149" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B22" s="127" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C22" s="133" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D22" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E22" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F22" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G22" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H22" s="135" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I22" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4583,22 +4603,22 @@
       <c r="A23" s="131"/>
       <c r="B23" s="140"/>
       <c r="C23" s="133" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D23" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E23" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F23" s="142" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G23" s="142" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H23" s="85" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I23" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4643,7 +4663,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="120" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B24" s="121"/>
       <c r="C24" s="121"/>
@@ -4685,28 +4705,28 @@
     </row>
     <row r="25" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="126" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B25" s="127" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C25" s="128" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D25" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E25" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F25" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G25" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H25" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I25" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4748,22 +4768,22 @@
       <c r="A26" s="131"/>
       <c r="B26" s="132"/>
       <c r="C26" s="133" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D26" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E26" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F26" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G26" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H26" s="135" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I26" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4803,28 +4823,28 @@
     </row>
     <row r="27" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="126" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B27" s="127" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C27" s="133" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D27" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E27" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F27" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G27" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H27" s="135" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I27" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4866,10 +4886,10 @@
       <c r="A28" s="131"/>
       <c r="B28" s="132"/>
       <c r="C28" s="133" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D28" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E28" s="129"/>
       <c r="F28" s="134"/>
@@ -4912,28 +4932,28 @@
     </row>
     <row r="29" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="126" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B29" s="127" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C29" s="133" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D29" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E29" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F29" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G29" s="134" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H29" s="135" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I29" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4975,10 +4995,10 @@
       <c r="A30" s="149"/>
       <c r="B30" s="150"/>
       <c r="C30" s="133" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D30" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E30" s="129"/>
       <c r="F30" s="134"/>
@@ -5023,10 +5043,10 @@
       <c r="A31" s="149"/>
       <c r="B31" s="150"/>
       <c r="C31" s="133" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D31" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E31" s="129"/>
       <c r="F31" s="134"/>
@@ -5071,10 +5091,10 @@
       <c r="A32" s="131"/>
       <c r="B32" s="132"/>
       <c r="C32" s="133" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D32" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E32" s="129"/>
       <c r="F32" s="134"/>
@@ -5117,16 +5137,16 @@
     </row>
     <row r="33" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="149" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B33" s="150" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C33" s="151" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D33" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E33" s="129"/>
       <c r="F33" s="134"/>
@@ -5171,10 +5191,10 @@
       <c r="A34" s="152"/>
       <c r="B34" s="140"/>
       <c r="C34" s="151" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E34" s="129"/>
       <c r="F34" s="142"/>
@@ -5222,7 +5242,7 @@
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="120" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B35" s="121"/>
       <c r="C35" s="121"/>
@@ -5265,16 +5285,16 @@
     </row>
     <row r="36" ht="27" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="126" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B36" s="127" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C36" s="153" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D36" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E36" s="129"/>
       <c r="F36" s="130"/>
@@ -5320,10 +5340,10 @@
       <c r="A37" s="131"/>
       <c r="B37" s="132"/>
       <c r="C37" s="155" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D37" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E37" s="129"/>
       <c r="F37" s="130"/>
@@ -5367,28 +5387,28 @@
     </row>
     <row r="38" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="126" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B38" s="127" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C38" s="155" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D38" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E38" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F38" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G38" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H38" s="154" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I38" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5431,10 +5451,10 @@
       <c r="A39" s="149"/>
       <c r="B39" s="150"/>
       <c r="C39" s="153" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D39" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E39" s="129"/>
       <c r="F39" s="130"/>
@@ -5480,22 +5500,22 @@
       <c r="A40" s="149"/>
       <c r="B40" s="150"/>
       <c r="C40" s="155" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D40" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E40" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F40" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G40" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H40" s="154" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I40" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5536,16 +5556,16 @@
     </row>
     <row r="41" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="126" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B41" s="127" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C41" s="155" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D41" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E41" s="129"/>
       <c r="F41" s="130"/>
@@ -5591,10 +5611,10 @@
       <c r="A42" s="152"/>
       <c r="B42" s="140"/>
       <c r="C42" s="156" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D42" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E42" s="129"/>
       <c r="F42" s="142"/>
@@ -5642,7 +5662,7 @@
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="157" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B43" s="158"/>
       <c r="C43" s="146"/>
@@ -5685,28 +5705,28 @@
     </row>
     <row r="44" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="126" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B44" s="127" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C44" s="155" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D44" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E44" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F44" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G44" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H44" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I44" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5749,22 +5769,22 @@
       <c r="A45" s="131"/>
       <c r="B45" s="132"/>
       <c r="C45" s="155" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D45" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E45" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F45" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G45" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H45" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I45" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5805,16 +5825,16 @@
     </row>
     <row r="46" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="131" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B46" s="159" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C46" s="155" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D46" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E46" s="129"/>
       <c r="F46" s="130"/>
@@ -5858,16 +5878,16 @@
     </row>
     <row r="47" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="126" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B47" s="127" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C47" s="155" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D47" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E47" s="129"/>
       <c r="F47" s="130"/>
@@ -5913,10 +5933,10 @@
       <c r="A48" s="131"/>
       <c r="B48" s="132"/>
       <c r="C48" s="155" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D48" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E48" s="129"/>
       <c r="F48" s="130"/>
@@ -5960,16 +5980,16 @@
     </row>
     <row r="49" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="126" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B49" s="127" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C49" s="155" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="D49" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E49" s="129"/>
       <c r="F49" s="130"/>
@@ -6015,10 +6035,10 @@
       <c r="A50" s="149"/>
       <c r="B50" s="150"/>
       <c r="C50" s="155" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D50" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E50" s="129"/>
       <c r="F50" s="130"/>
@@ -6064,22 +6084,22 @@
       <c r="A51" s="149"/>
       <c r="B51" s="150"/>
       <c r="C51" s="155" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D51" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E51" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F51" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G51" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H51" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I51" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6122,10 +6142,10 @@
       <c r="A52" s="149"/>
       <c r="B52" s="150"/>
       <c r="C52" s="155" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D52" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E52" s="129"/>
       <c r="F52" s="130"/>
@@ -6171,10 +6191,10 @@
       <c r="A53" s="131"/>
       <c r="B53" s="132"/>
       <c r="C53" s="155" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D53" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E53" s="129"/>
       <c r="F53" s="130"/>
@@ -6218,28 +6238,28 @@
     </row>
     <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="126" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B54" s="127" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C54" s="155" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D54" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E54" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F54" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G54" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H54" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I54" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6282,22 +6302,22 @@
       <c r="A55" s="149"/>
       <c r="B55" s="150"/>
       <c r="C55" s="155" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D55" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E55" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F55" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G55" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H55" s="70" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I55" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6340,10 +6360,10 @@
       <c r="A56" s="131"/>
       <c r="B56" s="132"/>
       <c r="C56" s="155" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D56" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E56" s="129"/>
       <c r="F56" s="130"/>
@@ -6387,16 +6407,16 @@
     </row>
     <row r="57" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="126" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B57" s="127" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C57" s="155" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D57" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E57" s="129"/>
       <c r="F57" s="130"/>
@@ -6442,10 +6462,10 @@
       <c r="A58" s="152"/>
       <c r="B58" s="140"/>
       <c r="C58" s="160" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D58" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E58" s="129"/>
       <c r="F58" s="134"/>
@@ -6493,7 +6513,7 @@
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="161" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B59" s="162"/>
       <c r="C59" s="121"/>
@@ -6536,16 +6556,16 @@
     </row>
     <row r="60" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="126" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B60" s="127" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C60" s="128" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D60" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E60" s="129"/>
       <c r="F60" s="130"/>
@@ -6591,10 +6611,10 @@
       <c r="A61" s="149"/>
       <c r="B61" s="150"/>
       <c r="C61" s="128" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D61" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E61" s="129"/>
       <c r="F61" s="130"/>
@@ -6640,10 +6660,10 @@
       <c r="A62" s="149"/>
       <c r="B62" s="150"/>
       <c r="C62" s="128" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D62" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E62" s="129"/>
       <c r="F62" s="130"/>
@@ -6689,10 +6709,10 @@
       <c r="A63" s="149"/>
       <c r="B63" s="150"/>
       <c r="C63" s="128" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D63" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E63" s="129"/>
       <c r="F63" s="130"/>
@@ -6738,10 +6758,10 @@
       <c r="A64" s="131"/>
       <c r="B64" s="132"/>
       <c r="C64" s="128" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D64" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E64" s="129"/>
       <c r="F64" s="130"/>
@@ -6785,28 +6805,28 @@
     </row>
     <row r="65" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A65" s="126" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B65" s="127" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C65" s="128" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D65" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E65" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F65" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G65" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H65" s="163" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I65" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6849,22 +6869,22 @@
       <c r="A66" s="149"/>
       <c r="B66" s="150"/>
       <c r="C66" s="128" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D66" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E66" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F66" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G66" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H66" s="163" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I66" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6907,10 +6927,10 @@
       <c r="A67" s="131"/>
       <c r="B67" s="132"/>
       <c r="C67" s="128" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D67" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E67" s="129"/>
       <c r="F67" s="130"/>
@@ -6954,16 +6974,16 @@
     </row>
     <row r="68" ht="24.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A68" s="126" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B68" s="127" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C68" s="148" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D68" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E68" s="129"/>
       <c r="F68" s="130"/>
@@ -7009,10 +7029,10 @@
       <c r="A69" s="131"/>
       <c r="B69" s="132"/>
       <c r="C69" s="128" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D69" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E69" s="129"/>
       <c r="F69" s="130"/>
@@ -7056,28 +7076,28 @@
     </row>
     <row r="70" ht="24.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70" s="164" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B70" s="165" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C70" s="148" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D70" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E70" s="129" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F70" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G70" s="130" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H70" s="163" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I70" s="123" t="str">
         <f t="shared" ref="I70:I74" si="39">(IF(COUNTA(D70:H70)&gt;1,"◄",""))</f>
@@ -7118,16 +7138,16 @@
     </row>
     <row r="71" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71" s="126" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B71" s="127" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C71" s="128" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D71" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E71" s="129"/>
       <c r="F71" s="130"/>
@@ -7173,7 +7193,7 @@
       <c r="A72" s="131"/>
       <c r="B72" s="132"/>
       <c r="C72" s="166" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D72" s="129"/>
       <c r="E72" s="129"/>
@@ -7218,16 +7238,16 @@
     </row>
     <row r="73" ht="13.7" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A73" s="126" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B73" s="167" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C73" s="166" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D73" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E73" s="129"/>
       <c r="F73" s="130"/>
@@ -7273,10 +7293,10 @@
       <c r="A74" s="152"/>
       <c r="B74" s="168"/>
       <c r="C74" s="156" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D74" s="129" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E74" s="129"/>
       <c r="F74" s="142"/>
@@ -7332,7 +7352,7 @@
       <c r="G75" s="170"/>
       <c r="H75" s="170"/>
       <c r="I75" s="171" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="J75" s="143"/>
       <c r="L75" s="144"/>
@@ -7347,7 +7367,7 @@
     </row>
     <row r="76" spans="3:18" x14ac:dyDescent="0.25">
       <c r="C76" s="172" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E76" s="173">
         <f>P4*K4+P35*K35+P43*K43+P59*K59+P15*K15+P24*K24</f>
@@ -7381,7 +7401,7 @@
     </row>
     <row r="77" ht="13.5" customHeight="1" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C77" s="177" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="E77" s="178" t="str">
         <f>IF(E76&lt;30%,"!",IF(Q76&lt;&gt;0,"",(IF(N76&lt;&gt;0,(M4*K4+M15*K15+M24*K24+M35*K35+M43*K43+M59*K59)/(K4*N4+K15*N15+K24*N24+K35*N35+K43*N43+K59*N59),0))))</f>
@@ -7389,22 +7409,22 @@
       </c>
       <c r="F77" s="178"/>
       <c r="G77" s="179" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="H77" s="179"/>
       <c r="I77" s="171" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="J77" s="180"/>
     </row>
     <row r="78" ht="23.25" customHeight="1" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C78" s="181" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E78" s="182"/>
       <c r="F78" s="183"/>
       <c r="G78" s="184" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="H78" s="185"/>
       <c r="I78" s="171"/>
@@ -7412,24 +7432,24 @@
     </row>
     <row r="79" ht="21.75" customHeight="1" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C79" s="181" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="E79" s="186">
         <f>IF(Q76&lt;&gt;0,"",E78*3)</f>
       </c>
       <c r="F79" s="187"/>
       <c r="G79" s="188" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="H79" s="189"/>
       <c r="I79" s="171" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="J79" s="180"/>
     </row>
     <row r="80" ht="17.45" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="190" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B80" s="190"/>
       <c r="C80" s="190"/>
@@ -7443,7 +7463,7 @@
     </row>
     <row r="81" ht="13.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="192" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B81" s="193"/>
       <c r="C81" s="193"/>
@@ -7453,13 +7473,13 @@
       <c r="G81" s="193"/>
       <c r="H81" s="193"/>
       <c r="I81" s="171" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="J81" s="194"/>
     </row>
     <row r="82" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="195" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B82" s="196"/>
       <c r="C82" s="197" t="str">
@@ -7500,15 +7520,15 @@
     </row>
     <row r="85" ht="12.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="206" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B85" s="207"/>
       <c r="C85" s="208" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D85" s="114"/>
       <c r="E85" s="209" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="F85" s="210"/>
       <c r="G85" s="210"/>
@@ -7518,7 +7538,7 @@
     </row>
     <row r="86" ht="39.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="211" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B86" s="212"/>
       <c r="C86" s="70"/>

</xml_diff>

<commit_message>
Mise à jour des réponses pour question1
</commit_message>
<xml_diff>
--- a/fichier_eleves/J1.xlsx
+++ b/fichier_eleves/J1.xlsx
@@ -504,10 +504,10 @@
     <t>Les différents documents liés : au conducteur, véhicule, marchandise transportée, réglementation figurent sans omission dans la pochette à constituer.</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>X</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Les documents présents sont valides.</t>
@@ -4386,16 +4386,16 @@
         <v>19</v>
       </c>
       <c r="E19" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F19" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G19" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H19" s="135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I19" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4495,16 +4495,16 @@
         <v>19</v>
       </c>
       <c r="E21" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F21" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G21" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H21" s="135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I21" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4552,16 +4552,16 @@
         <v>19</v>
       </c>
       <c r="E22" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F22" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G22" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H22" s="135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I22" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4609,16 +4609,16 @@
         <v>19</v>
       </c>
       <c r="E23" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F23" s="142" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G23" s="142" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H23" s="85" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I23" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4717,16 +4717,16 @@
         <v>19</v>
       </c>
       <c r="E25" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F25" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G25" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H25" s="70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I25" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4774,16 +4774,16 @@
         <v>19</v>
       </c>
       <c r="E26" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F26" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G26" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H26" s="135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I26" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4835,16 +4835,16 @@
         <v>19</v>
       </c>
       <c r="E27" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F27" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G27" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H27" s="135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I27" s="123" t="str">
         <f t="shared" si="7"/>
@@ -4944,16 +4944,16 @@
         <v>19</v>
       </c>
       <c r="E29" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F29" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G29" s="134" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H29" s="135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I29" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5399,16 +5399,16 @@
         <v>19</v>
       </c>
       <c r="E38" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F38" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G38" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H38" s="154" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I38" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5506,16 +5506,16 @@
         <v>19</v>
       </c>
       <c r="E40" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F40" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G40" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H40" s="154" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I40" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5717,16 +5717,16 @@
         <v>19</v>
       </c>
       <c r="E44" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F44" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G44" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H44" s="70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I44" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5775,16 +5775,16 @@
         <v>19</v>
       </c>
       <c r="E45" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F45" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G45" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H45" s="70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I45" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6090,16 +6090,16 @@
         <v>19</v>
       </c>
       <c r="E51" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F51" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G51" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H51" s="70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I51" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6250,16 +6250,16 @@
         <v>19</v>
       </c>
       <c r="E54" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F54" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G54" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H54" s="70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I54" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6308,16 +6308,16 @@
         <v>19</v>
       </c>
       <c r="E55" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F55" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G55" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H55" s="70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I55" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6817,16 +6817,16 @@
         <v>19</v>
       </c>
       <c r="E65" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F65" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G65" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H65" s="163" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I65" s="123" t="str">
         <f t="shared" si="7"/>
@@ -6875,16 +6875,16 @@
         <v>19</v>
       </c>
       <c r="E66" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F66" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G66" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H66" s="163" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I66" s="123" t="str">
         <f t="shared" si="7"/>
@@ -7088,16 +7088,16 @@
         <v>19</v>
       </c>
       <c r="E70" s="129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F70" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G70" s="130" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H70" s="163" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I70" s="123" t="str">
         <f t="shared" ref="I70:I74" si="39">(IF(COUNTA(D70:H70)&gt;1,"◄",""))</f>

</xml_diff>

<commit_message>
Mise à jour des réponses pour question8
</commit_message>
<xml_diff>
--- a/fichier_eleves/J1.xlsx
+++ b/fichier_eleves/J1.xlsx
@@ -5726,7 +5726,7 @@
         <v>112</v>
       </c>
       <c r="H44" s="70" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I44" s="123" t="str">
         <f t="shared" si="7"/>
@@ -5784,7 +5784,7 @@
         <v>112</v>
       </c>
       <c r="H45" s="70" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I45" s="123" t="str">
         <f t="shared" si="7"/>

</xml_diff>